<commit_message>
ui and api test cases are created
</commit_message>
<xml_diff>
--- a/Manual Testing Report/Manual_Testing_Report.xlsx
+++ b/Manual Testing Report/Manual_Testing_Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\==Placements==\Capgemini\sprint\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\==Projects==\Selenium_Python_Advanced_Capstone\Manual Testing Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C29DB6-4924-4222-8F29-56976A0116F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0552F58-FF0A-42A4-AA74-6ED5379CC8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Guidance &amp; Instructions" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="411">
   <si>
     <t>MANUAL TESTING DOCUMENTATION GUIDE</t>
   </si>
@@ -1233,15 +1233,6 @@
   </si>
   <si>
     <t>When a note is created successfully, the application does not display the expected success confirmation message to the user</t>
-  </si>
-  <si>
-    <t>Large description validation issue</t>
-  </si>
-  <si>
-    <t>Application does not handle large note descriptions correctly and accepts input only between 4 to 1000 characters without proper validation messaging</t>
-  </si>
-  <si>
-    <t>Validation limit needs clarification</t>
   </si>
   <si>
     <t>Yes API returns status code 200</t>
@@ -1368,7 +1359,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1404,12 +1395,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1435,9 +1450,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1447,9 +1459,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2054,7 +2082,7 @@
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2086,7 +2114,7 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2178,7 +2206,7 @@
       <c r="A25" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="16">
         <v>46148</v>
       </c>
     </row>
@@ -2551,7 +2579,7 @@
         <v>102</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2580,7 +2608,7 @@
         <v>102</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2609,7 +2637,7 @@
         <v>102</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2638,7 +2666,7 @@
         <v>107</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2667,7 +2695,7 @@
         <v>102</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
@@ -2686,7 +2714,7 @@
         <v>184</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="F7" s="10" t="s">
         <v>224</v>
@@ -2698,7 +2726,7 @@
         <v>102</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2727,7 +2755,7 @@
         <v>107</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2756,7 +2784,7 @@
         <v>102</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2785,7 +2813,7 @@
         <v>107</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2802,7 +2830,7 @@
         <v>184</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>237</v>
@@ -2814,7 +2842,7 @@
         <v>102</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2837,13 +2865,13 @@
         <v>242</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2866,13 +2894,13 @@
         <v>245</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2901,7 +2929,7 @@
         <v>102</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
@@ -2930,7 +2958,7 @@
         <v>102</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2950,10 +2978,10 @@
         <v>275</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>102</v>
@@ -2976,7 +3004,7 @@
         <v>193</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>260</v>
@@ -3011,13 +3039,13 @@
         <v>264</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
@@ -3040,13 +3068,13 @@
         <v>267</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>107</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
@@ -3098,13 +3126,13 @@
         <v>271</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>107</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -3405,7 +3433,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="14"/>
+      <c r="A23" s="13"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
@@ -3472,7 +3500,7 @@
       <c r="D2" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E2" s="15">
+      <c r="E2" s="14">
         <v>45417</v>
       </c>
       <c r="F2" s="10" t="s">
@@ -3496,7 +3524,7 @@
       <c r="D3" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E3" s="15">
+      <c r="E3" s="14">
         <v>45417</v>
       </c>
       <c r="F3" s="10" t="s">
@@ -3520,7 +3548,7 @@
       <c r="D4" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="14">
         <v>45417</v>
       </c>
       <c r="F4" s="10" t="s">
@@ -3544,7 +3572,7 @@
       <c r="D5" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="14">
         <v>45417</v>
       </c>
       <c r="F5" s="10" t="s">
@@ -3568,7 +3596,7 @@
       <c r="D6" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="14">
         <v>45417</v>
       </c>
       <c r="F6" s="10" t="s">
@@ -3592,7 +3620,7 @@
       <c r="D7" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="14">
         <v>45418</v>
       </c>
       <c r="F7" s="10" t="s">
@@ -3616,7 +3644,7 @@
       <c r="D8" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="14">
         <v>45418</v>
       </c>
       <c r="F8" s="10" t="s">
@@ -3642,7 +3670,7 @@
       <c r="D9" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="14">
         <v>45418</v>
       </c>
       <c r="F9" s="10" t="s">
@@ -3666,7 +3694,7 @@
       <c r="D10" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="14">
         <v>45418</v>
       </c>
       <c r="F10" s="10" t="s">
@@ -3692,7 +3720,7 @@
       <c r="D11" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="14">
         <v>45418</v>
       </c>
       <c r="F11" s="10" t="s">
@@ -3716,7 +3744,7 @@
       <c r="D12" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="14">
         <v>45418</v>
       </c>
       <c r="F12" s="10" t="s">
@@ -3740,7 +3768,7 @@
       <c r="D13" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="14">
         <v>45418</v>
       </c>
       <c r="F13" s="10" t="s">
@@ -3764,7 +3792,7 @@
       <c r="D14" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="14">
         <v>45418</v>
       </c>
       <c r="F14" s="10" t="s">
@@ -3788,7 +3816,7 @@
       <c r="D15" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="14">
         <v>45418</v>
       </c>
       <c r="F15" s="10" t="s">
@@ -3812,7 +3840,7 @@
       <c r="D16" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="14">
         <v>45418</v>
       </c>
       <c r="F16" s="10" t="s">
@@ -3836,7 +3864,7 @@
       <c r="D17" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="14">
         <v>45418</v>
       </c>
       <c r="F17" s="10" t="s">
@@ -3860,7 +3888,7 @@
       <c r="D18" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="14">
         <v>45418</v>
       </c>
       <c r="F18" s="10" t="s">
@@ -3884,7 +3912,7 @@
       <c r="D19" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="14">
         <v>45418</v>
       </c>
       <c r="F19" s="10" t="s">
@@ -3908,7 +3936,7 @@
       <c r="D20" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="14">
         <v>45418</v>
       </c>
       <c r="F20" s="10" t="s">
@@ -3932,7 +3960,7 @@
       <c r="D21" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="14">
         <v>45418</v>
       </c>
       <c r="F21" s="10" t="s">
@@ -4141,7 +4169,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4191,7 +4219,7 @@
       <c r="A2" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="19" t="s">
         <v>147</v>
       </c>
       <c r="C2" s="10" t="s">
@@ -4212,62 +4240,57 @@
       <c r="H2" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="I2" s="15">
+      <c r="I2" s="14">
         <v>45418</v>
       </c>
       <c r="J2" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="K2" s="11"/>
+      <c r="K2" s="23"/>
       <c r="L2" s="11"/>
     </row>
-    <row r="3" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>398</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="I3" s="15">
-        <v>45418</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="K3" s="13"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="22"/>
       <c r="L3" s="9"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="13"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="22"/>
       <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implemented manual testing and automation testing
</commit_message>
<xml_diff>
--- a/Manual Testing Report/Manual_Testing_Report.xlsx
+++ b/Manual Testing Report/Manual_Testing_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\==Projects==\Selenium_Python_Advanced_Capstone\Manual Testing Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0552F58-FF0A-42A4-AA74-6ED5379CC8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DF45C4-D6FF-434E-9A9F-40BA9507A06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Guidance &amp; Instructions" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="410">
   <si>
     <t>MANUAL TESTING DOCUMENTATION GUIDE</t>
   </si>
@@ -348,9 +348,6 @@
   </si>
   <si>
     <t>High</t>
-  </si>
-  <si>
-    <t>Not Started</t>
   </si>
   <si>
     <t>TC-002</t>
@@ -1424,7 +1421,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1460,24 +1457,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2072,17 +2062,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="21"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2114,7 +2104,7 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2288,13 +2278,13 @@
         <v>90</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>181</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -2302,13 +2292,13 @@
         <v>92</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>202</v>
-      </c>
       <c r="D3" s="10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -2316,125 +2306,125 @@
         <v>93</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>206</v>
-      </c>
       <c r="D6" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>189</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>191</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>194</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>198</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -2544,7 +2534,7 @@
         <v>97</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>98</v>
@@ -2567,572 +2557,572 @@
         <v>91</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>359</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>215</v>
-      </c>
       <c r="G3" s="10" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>360</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>218</v>
-      </c>
       <c r="G5" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="F6" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>221</v>
-      </c>
       <c r="G6" s="10" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
     </row>
     <row r="7" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>404</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>224</v>
-      </c>
       <c r="G7" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="F8" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>227</v>
-      </c>
       <c r="G8" s="10" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="E9" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>231</v>
-      </c>
       <c r="G9" s="10" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C10" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="E10" s="10" t="s">
+      <c r="G10" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>370</v>
-      </c>
       <c r="H10" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>403</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>237</v>
-      </c>
       <c r="G11" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>242</v>
-      </c>
       <c r="G12" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>273</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>245</v>
-      </c>
       <c r="G13" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="D14" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>248</v>
-      </c>
       <c r="G14" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="D15" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>251</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>252</v>
-      </c>
       <c r="G15" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F16" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="G16" s="10" t="s">
         <v>407</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>408</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>103</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>259</v>
       </c>
-      <c r="D17" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>405</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>260</v>
-      </c>
       <c r="G17" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>103</v>
+        <v>405</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C18" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E18" s="10" t="s">
+      <c r="F18" s="10" t="s">
         <v>263</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>264</v>
-      </c>
       <c r="G18" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C19" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="E19" s="10" t="s">
+      <c r="F19" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>267</v>
-      </c>
       <c r="G19" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C20" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>194</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>269</v>
-      </c>
       <c r="G20" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>103</v>
+        <v>405</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C21" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="F21" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>271</v>
-      </c>
       <c r="G21" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -3154,282 +3144,282 @@
   <sheetData>
     <row r="1" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>278</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>343</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="10" t="s">
         <v>344</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>292</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>341</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>294</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>342</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>296</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>371</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>298</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>291</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>300</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>291</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>301</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="10" t="s">
         <v>303</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>306</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
         <v>310</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>314</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>321</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>324</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>325</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="D17" s="10" t="s">
         <v>328</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B18" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>331</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B19" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>334</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B20" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>337</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -3466,25 +3456,25 @@
         <v>94</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>95</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -3492,483 +3482,481 @@
         <v>100</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>101</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E2" s="14">
         <v>45417</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E3" s="14">
         <v>45417</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E4" s="14">
         <v>45417</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="10" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E5" s="14">
         <v>45417</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E6" s="14">
         <v>45417</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="D7" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E7" s="14">
         <v>45418</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E8" s="14">
         <v>45418</v>
       </c>
       <c r="F8" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>129</v>
-      </c>
       <c r="H8" s="10" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="D9" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E9" s="14">
         <v>45418</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G9" s="10"/>
       <c r="H9" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E10" s="14">
         <v>45418</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>145</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="G10" s="10"/>
       <c r="H10" s="10" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="D11" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E11" s="14">
         <v>45418</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G11" s="10"/>
       <c r="H11" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E12" s="14">
         <v>45418</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G12" s="10"/>
       <c r="H12" s="10" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="D13" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E13" s="14">
         <v>45418</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E14" s="14">
         <v>45418</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G14" s="10"/>
       <c r="H14" s="10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E15" s="14">
         <v>45418</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G15" s="10"/>
       <c r="H15" s="10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>257</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E16" s="14">
         <v>45418</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G16" s="10"/>
       <c r="H16" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>259</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E17" s="14">
         <v>45418</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G17" s="10"/>
       <c r="H17" s="10" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B18" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>262</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E18" s="14">
         <v>45418</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B19" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>264</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E19" s="14">
         <v>45418</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G19" s="10"/>
       <c r="H19" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B20" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E20" s="14">
         <v>45418</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G20" s="10"/>
       <c r="H20" s="10" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B21" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E21" s="14">
         <v>45418</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>357</v>
+        <v>125</v>
       </c>
       <c r="G21" s="10"/>
       <c r="H21" s="10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
   </sheetData>
@@ -3989,16 +3977,16 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>94</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>99</v>
@@ -4006,155 +3994,155 @@
     </row>
     <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>377</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="10" t="s">
         <v>378</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>379</v>
-      </c>
       <c r="D2" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E2" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
+        <v>379</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>373</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>381</v>
-      </c>
       <c r="D3" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>382</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>383</v>
-      </c>
       <c r="D4" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>384</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>374</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>385</v>
-      </c>
       <c r="D5" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
+        <v>385</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>386</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>387</v>
-      </c>
       <c r="D6" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D7" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
+        <v>388</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>390</v>
-      </c>
       <c r="D8" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>391</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>392</v>
-      </c>
       <c r="D9" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>393</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C10" s="10" t="s">
         <v>394</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>395</v>
-      </c>
       <c r="D10" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -4169,7 +4157,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4185,19 +4173,19 @@
   <sheetData>
     <row r="1" spans="1:12" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>94</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>138</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>139</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>98</v>
@@ -4206,91 +4194,80 @@
         <v>99</v>
       </c>
       <c r="H1" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>141</v>
-      </c>
       <c r="J1" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>147</v>
+        <v>128</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>146</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>396</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>397</v>
-      </c>
       <c r="E2" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>102</v>
       </c>
       <c r="G2" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="H2" s="10" t="s">
         <v>142</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>143</v>
       </c>
       <c r="I2" s="14">
         <v>45418</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="K2" s="23"/>
+        <v>143</v>
+      </c>
+      <c r="K2" s="11"/>
       <c r="L2" s="11"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="22"/>
+        <v>144</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="19"/>
       <c r="L3" s="9"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="15"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="22"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="19"/>
       <c r="L4" s="9"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
-      <c r="K5" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4307,14 +4284,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="17" t="s">
-        <v>148</v>
-      </c>
-      <c r="B1" s="18"/>
+      <c r="A1" s="20" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="21"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -4324,15 +4301,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B6" t="s">
         <v>59</v>
@@ -4345,12 +4322,12 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B10">
         <v>20</v>
@@ -4358,7 +4335,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B11">
         <v>20</v>
@@ -4366,7 +4343,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B12">
         <v>18</v>
@@ -4374,7 +4351,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -4382,7 +4359,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B14" s="8">
         <f>B12/B11*100</f>
@@ -4391,12 +4368,12 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -4404,7 +4381,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -4412,7 +4389,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -4420,7 +4397,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -4428,7 +4405,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -4436,7 +4413,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B22">
         <v>2</v>
@@ -4444,7 +4421,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -4452,36 +4429,36 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B26" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>167</v>
+      </c>
+      <c r="B27" t="s">
         <v>168</v>
-      </c>
-      <c r="B27" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>169</v>
+      </c>
+      <c r="B28" t="s">
         <v>170</v>
-      </c>
-      <c r="B28" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated code in pages
</commit_message>
<xml_diff>
--- a/Manual Testing Report/Manual_Testing_Report.xlsx
+++ b/Manual Testing Report/Manual_Testing_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\==Projects==\Selenium_Python_Advanced_Capstone\Manual Testing Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DF45C4-D6FF-434E-9A9F-40BA9507A06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72CBAABB-690B-4EE8-B97B-40DC655B4120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0. Guidance &amp; Instructions" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="402">
   <si>
     <t>MANUAL TESTING DOCUMENTATION GUIDE</t>
   </si>
@@ -473,9 +473,6 @@
     <t>Needs investigation</t>
   </si>
   <si>
-    <t>DEF-002</t>
-  </si>
-  <si>
     <t>TC-005</t>
   </si>
   <si>
@@ -911,9 +908,6 @@
     <t>Used for invalid password validation</t>
   </si>
   <si>
-    <t>""</t>
-  </si>
-  <si>
     <t>Valid Note Title</t>
   </si>
   <si>
@@ -932,18 +926,6 @@
     <t>Used for large text validation</t>
   </si>
   <si>
-    <t>Empty Note Title</t>
-  </si>
-  <si>
-    <t>Used for empty note title validation</t>
-  </si>
-  <si>
-    <t>Empty Note Description</t>
-  </si>
-  <si>
-    <t>Used for empty description validation</t>
-  </si>
-  <si>
     <t>API Auth Token</t>
   </si>
   <si>
@@ -977,27 +959,12 @@
     <t>TD-015</t>
   </si>
   <si>
-    <t>Invalid HTTP Method</t>
-  </si>
-  <si>
-    <t>PATCH /notes</t>
-  </si>
-  <si>
-    <t>Used for invalid HTTP method validation</t>
-  </si>
-  <si>
     <t>TD-016</t>
   </si>
   <si>
     <t>TD-017</t>
   </si>
   <si>
-    <t>TD-018</t>
-  </si>
-  <si>
-    <t>TD-019</t>
-  </si>
-  <si>
     <t>Invalid Note ID</t>
   </si>
   <si>
@@ -1007,9 +974,6 @@
     <t>Used for invalid note deletion validation</t>
   </si>
   <si>
-    <t>TD-020</t>
-  </si>
-  <si>
     <t>UI Created Note Data</t>
   </si>
   <si>
@@ -1269,6 +1233,18 @@
   </si>
   <si>
     <t>K.Sathwik</t>
+  </si>
+  <si>
+    <t>Empty fields for Note creation Note Title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Title :""                                                 Description:""                                                                                                                                                  </t>
+  </si>
+  <si>
+    <t>Used for empty note title and description validation</t>
+  </si>
+  <si>
+    <t>TD-005</t>
   </si>
 </sst>
 </file>
@@ -1356,7 +1332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1374,43 +1350,6 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -1453,21 +1392,19 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2062,17 +1999,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="21"/>
+      <c r="B1" s="18"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -2104,7 +2041,7 @@
         <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -2196,7 +2133,7 @@
       <c r="A25" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="16">
+      <c r="B25" s="15">
         <v>46148</v>
       </c>
     </row>
@@ -2278,13 +2215,13 @@
         <v>90</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>180</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -2292,13 +2229,13 @@
         <v>92</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>201</v>
-      </c>
       <c r="D3" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -2306,125 +2243,125 @@
         <v>93</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>205</v>
-      </c>
       <c r="D6" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>188</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>190</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>193</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>197</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -2534,7 +2471,7 @@
         <v>97</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>98</v>
@@ -2557,19 +2494,19 @@
         <v>91</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2580,25 +2517,25 @@
         <v>92</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>358</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>214</v>
-      </c>
       <c r="G3" s="10" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2612,22 +2549,22 @@
         <v>104</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
@@ -2638,491 +2575,491 @@
         <v>92</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>347</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>359</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>217</v>
-      </c>
       <c r="G5" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>106</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C6" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="F6" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>220</v>
-      </c>
       <c r="G6" s="10" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
     </row>
     <row r="7" spans="1:11" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C7" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>391</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>403</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>223</v>
-      </c>
       <c r="G7" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C8" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="E8" s="10" t="s">
+      <c r="F8" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>226</v>
-      </c>
       <c r="G8" s="10" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>106</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="D9" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="E9" s="10" t="s">
+      <c r="F9" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>230</v>
-      </c>
       <c r="G9" s="10" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>93</v>
       </c>
       <c r="C10" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>233</v>
-      </c>
       <c r="G10" s="10" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>106</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="D11" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>402</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>236</v>
-      </c>
       <c r="G11" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="C12" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>241</v>
-      </c>
       <c r="G12" s="10" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>244</v>
-      </c>
       <c r="G13" s="10" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="D14" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>273</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>247</v>
-      </c>
       <c r="G14" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="D15" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="D15" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>251</v>
-      </c>
       <c r="G15" s="10" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="D17" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>404</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>259</v>
-      </c>
       <c r="G17" s="10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C18" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="D18" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="E18" s="10" t="s">
+      <c r="F18" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>263</v>
-      </c>
       <c r="G18" s="10" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C19" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="E19" s="10" t="s">
+      <c r="F19" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>266</v>
-      </c>
       <c r="G19" s="10" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>106</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C20" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>268</v>
-      </c>
       <c r="G20" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>102</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C21" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="F21" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="D21" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>270</v>
-      </c>
       <c r="G21" s="10" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>106</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -3164,7 +3101,7 @@
         <v>112</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>113</v>
@@ -3175,13 +3112,13 @@
         <v>114</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -3189,13 +3126,13 @@
         <v>115</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -3203,116 +3140,116 @@
         <v>116</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>279</v>
+        <v>401</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>297</v>
+        <v>398</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>290</v>
+        <v>399</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>298</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>304</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>305</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>308</v>
@@ -3326,100 +3263,72 @@
     </row>
     <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>312</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>313</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>332</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>335</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>336</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
@@ -3509,7 +3418,7 @@
         <v>123</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>124</v>
@@ -3522,7 +3431,7 @@
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -3546,7 +3455,7 @@
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="10" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="58" x14ac:dyDescent="0.35">
@@ -3557,7 +3466,7 @@
         <v>123</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>124</v>
@@ -3570,18 +3479,18 @@
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>124</v>
@@ -3594,18 +3503,18 @@
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>124</v>
@@ -3614,22 +3523,22 @@
         <v>45418</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>124</v>
@@ -3644,18 +3553,18 @@
         <v>128</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>124</v>
@@ -3668,18 +3577,18 @@
       </c>
       <c r="G9" s="10"/>
       <c r="H9" s="10" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>124</v>
@@ -3692,18 +3601,18 @@
       </c>
       <c r="G10" s="10"/>
       <c r="H10" s="10" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>124</v>
@@ -3716,18 +3625,18 @@
       </c>
       <c r="G11" s="10"/>
       <c r="H11" s="10" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>124</v>
@@ -3740,18 +3649,18 @@
       </c>
       <c r="G12" s="10"/>
       <c r="H12" s="10" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>124</v>
@@ -3764,18 +3673,18 @@
       </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>124</v>
@@ -3788,18 +3697,18 @@
       </c>
       <c r="G14" s="10"/>
       <c r="H14" s="10" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>124</v>
@@ -3812,18 +3721,18 @@
       </c>
       <c r="G15" s="10"/>
       <c r="H15" s="10" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>124</v>
@@ -3836,18 +3745,18 @@
       </c>
       <c r="G16" s="10"/>
       <c r="H16" s="10" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>124</v>
@@ -3860,18 +3769,18 @@
       </c>
       <c r="G17" s="10"/>
       <c r="H17" s="10" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>124</v>
@@ -3884,18 +3793,18 @@
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="10" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>124</v>
@@ -3908,18 +3817,18 @@
       </c>
       <c r="G19" s="10"/>
       <c r="H19" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>124</v>
@@ -3932,18 +3841,18 @@
       </c>
       <c r="G20" s="10"/>
       <c r="H20" s="10" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>123</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>124</v>
@@ -3956,7 +3865,7 @@
       </c>
       <c r="G21" s="10"/>
       <c r="H21" s="10" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -3994,13 +3903,13 @@
     </row>
     <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="10" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>132</v>
@@ -4011,13 +3920,13 @@
     </row>
     <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>132</v>
@@ -4028,13 +3937,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="10" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>132</v>
@@ -4045,13 +3954,13 @@
     </row>
     <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>132</v>
@@ -4062,13 +3971,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="10" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>374</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>386</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>132</v>
@@ -4079,13 +3988,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>132</v>
@@ -4096,13 +4005,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>132</v>
@@ -4113,13 +4022,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>132</v>
@@ -4130,13 +4039,13 @@
     </row>
     <row r="10" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>132</v>
@@ -4157,7 +4066,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4207,14 +4116,14 @@
       <c r="A2" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>146</v>
+      <c r="B2" s="10" t="s">
+        <v>145</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>106</v>
@@ -4238,26 +4147,22 @@
       <c r="L2" s="11"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>231</v>
-      </c>
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
-      <c r="I3" s="19"/>
+      <c r="I3" s="16"/>
       <c r="J3" s="9"/>
-      <c r="K3" s="19"/>
+      <c r="K3" s="16"/>
       <c r="L3" s="9"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="15"/>
-      <c r="B4" s="18"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -4266,8 +4171,12 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
-      <c r="K4" s="19"/>
+      <c r="K4" s="16"/>
       <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4284,14 +4193,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="B1" s="21"/>
+      <c r="A1" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="18"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -4301,7 +4210,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B5" t="s">
         <v>123</v>
@@ -4309,7 +4218,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
         <v>59</v>
@@ -4322,12 +4231,12 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B10">
         <v>20</v>
@@ -4335,7 +4244,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B11">
         <v>20</v>
@@ -4343,7 +4252,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B12">
         <v>18</v>
@@ -4351,7 +4260,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B13">
         <v>2</v>
@@ -4359,7 +4268,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B14" s="8">
         <f>B12/B11*100</f>
@@ -4368,12 +4277,12 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B17">
         <v>2</v>
@@ -4381,7 +4290,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -4389,7 +4298,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -4397,7 +4306,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B20">
         <v>1</v>
@@ -4405,7 +4314,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -4413,7 +4322,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B22">
         <v>2</v>
@@ -4421,7 +4330,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -4429,12 +4338,12 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B26" t="s">
         <v>135</v>
@@ -4442,23 +4351,23 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B27" t="s">
         <v>167</v>
-      </c>
-      <c r="B27" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B28" t="s">
         <v>169</v>
-      </c>
-      <c r="B28" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>